<commit_message>
add new field to scitific forums
</commit_message>
<xml_diff>
--- a/resources/templates/scientific_forums/scientific_forums.xlsx
+++ b/resources/templates/scientific_forums/scientific_forums.xlsx
@@ -20,7 +20,7 @@
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="G1" authorId="0">
+    <comment ref="H1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -36,7 +36,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="0">
+    <comment ref="I1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="9">
   <si>
     <t>title_ka</t>
   </si>
@@ -65,22 +65,25 @@
     <t>title_en</t>
   </si>
   <si>
+    <t>scope</t>
+  </si>
+  <si>
+    <t>participation_role</t>
+  </si>
+  <si>
+    <t>end_date</t>
+  </si>
+  <si>
+    <t>start_date</t>
+  </si>
+  <si>
+    <t>participation_form_en</t>
+  </si>
+  <si>
     <t>participation_form_ka</t>
   </si>
   <si>
-    <t>participation_form_en</t>
-  </si>
-  <si>
-    <t>start_date</t>
-  </si>
-  <si>
-    <t>end_date</t>
-  </si>
-  <si>
-    <t>participation_role</t>
-  </si>
-  <si>
-    <t>scope</t>
+    <t>international_forum_publication</t>
   </si>
 </sst>
 </file>
@@ -420,10 +423,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -431,24 +434,27 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F1" t="s">
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1"/>
+        <v>3</v>
+      </c>
+      <c r="I1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>